<commit_message>
v0.9: tools, reactive blocks and active skills
</commit_message>
<xml_diff>
--- a/docs/balancing.xlsx
+++ b/docs/balancing.xlsx
@@ -18,6 +18,8 @@
     <sheet name="Dig times" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Battery" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Progress" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Tools &amp; skills" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Hazards" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,9 +31,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="234">
-  <si>
-    <t xml:space="preserve">Bolt &amp; Burrow — balancing sheet (v0.8.1)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="286">
+  <si>
+    <t xml:space="preserve">Bolt &amp; Burrow — balancing sheet (v0.9)</t>
   </si>
   <si>
     <t xml:space="preserve">A planning copy of the numbers in js/config.js. Changing this sheet does NOT change the game:</t>
@@ -73,6 +75,12 @@
     <t xml:space="preserve">Mods – every computer mod: shape, build cost, Flux to upgrade and how long the nano-bot takes to make it</t>
   </si>
   <si>
+    <t xml:space="preserve">Tools &amp; skills – tool prices and belt slots; active skills, their recharge times and battery cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hazards – how much sand, boulders, water and gas take when they hit you</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dig times – seconds to break each block with each arm tier ("—" = too hard for that tier)</t>
   </si>
   <si>
@@ -731,6 +739,156 @@
   </si>
   <si>
     <t xml:space="preserve">Relic rewards only. A negative running total is what you need to earn from block coins, caches and selling ore before that step (see Block coins). Mods are extra.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price (coins)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max per slot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full slot costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What it does</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blast charge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breaks a 3×3 area, even hard rock (you collect what breaks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Support beam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stops sand and boulders; keeps unstable rock within 1 block still</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lights a 7-block radius for 30 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grapple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swings across up to 3 blocks of chasm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belt slots</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base belt slots</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each tool type takes one slot. Pip buys tools back at full price.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery per use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recharge Lv 1 (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lv 2 (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lv 3 (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uses per minute at Lv 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drill Burst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scan Pulse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skills go in the computer's bottom row (opens with the Core Heart), one at a time. The nano-bot recharges them; upgrades use Flux like other mods.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hazard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery lost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ore lost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cave-in (unstable rock)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4 s shake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sets off unstable rock within 2.2 blocks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sand slide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3 s per block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slides toward the entrance into open space</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rolling boulder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6 s rumble, then 0.14 s per block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push one by walking into it for 0.3 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gas explosion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.9 s fuse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hits within 1.8 blocks; clears a 3×3 area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flood water</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2 per second</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2 s per block, 10 blocks a pocket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wading runs at 55% speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Shield blocks the whole hit. Every cave slopes toward its entrance, so sand and boulders move that way.</t>
   </si>
 </sst>
 </file>
@@ -1209,7 +1367,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1307,8 +1465,18 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1338,24 +1506,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B2" s="12" t="n">
         <f aca="false">Parts!D6</f>
@@ -1366,12 +1534,12 @@
         <v>-60</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B3" s="12" t="n">
         <f aca="false">Caves!O2</f>
@@ -1382,12 +1550,12 @@
         <v>-140</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C4" s="12" t="n">
         <f aca="false">Caves!N2</f>
@@ -1398,12 +1566,12 @@
         <v>160</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B5" s="12" t="n">
         <f aca="false">Parts!D3</f>
@@ -1414,12 +1582,12 @@
         <v>40</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B6" s="12" t="n">
         <f aca="false">Parts!D9</f>
@@ -1430,12 +1598,12 @@
         <v>-110</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">Caves!O3</f>
@@ -1449,7 +1617,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C8" s="12" t="n">
         <f aca="false">Caves!N3</f>
@@ -1460,12 +1628,12 @@
         <v>490</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">Parts!D7</f>
@@ -1476,12 +1644,12 @@
         <v>-410</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">Caves!O4</f>
@@ -1495,7 +1663,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">Caves!N4</f>
@@ -1506,12 +1674,546 @@
         <v>1090</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>233</v>
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" s="13" t="n">
+        <f aca="false">C2*D2</f>
+        <v>120</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" s="13" t="n">
+        <f aca="false">C3*D3</f>
+        <v>75</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" s="13" t="n">
+        <f aca="false">C4*D4</f>
+        <v>50</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <f aca="false">C5*D5</f>
+        <v>120</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <f aca="false">$B$12+0</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <f aca="false">$B$12+1</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <f aca="false">$B$12+2</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <f aca="false">60/K16</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <f aca="false">60/K17</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <f aca="false">60/K18</f>
+        <v>6.66666666666667</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="L19" s="15" t="n">
+        <f aca="false">60/K19</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -1540,244 +2242,244 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>1.2</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>45</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>80</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>60</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>160</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>54</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>0.5</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>0.4</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>1.8</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>0.25</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>0.3</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B22" s="4" t="n">
         <v>75</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1816,61 +2518,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1878,19 +2580,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E2" s="10" t="n">
         <v>0.06</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G2" s="10" t="n">
         <v>0.025</v>
@@ -1911,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="N2" s="11" t="n">
         <v>300</v>
@@ -1932,7 +2634,7 @@
         <v>160</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1940,19 +2642,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C3" s="9" t="n">
         <v>1.5</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E3" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G3" s="10" t="n">
         <v>0.03</v>
@@ -1973,7 +2675,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N3" s="11" t="n">
         <v>800</v>
@@ -1994,7 +2696,7 @@
         <v>240</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2002,19 +2704,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C4" s="9" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G4" s="10" t="n">
         <v>0.025</v>
@@ -2035,7 +2737,7 @@
         <v>3</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N4" s="11" t="n">
         <v>2000</v>
@@ -2056,17 +2758,17 @@
         <v>320</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2101,54 +2803,54 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D2" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>0</v>
@@ -2160,25 +2862,25 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D3" s="11" t="n">
         <v>120</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>3</v>
@@ -2190,25 +2892,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>1000</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>6</v>
@@ -2220,28 +2922,28 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I5" s="13" t="n">
         <f aca="false">SUM(D5:D5)</f>
@@ -2250,28 +2952,28 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>60</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="I6" s="13" t="n">
         <f aca="false">SUM(D5:D6)</f>
@@ -2280,28 +2982,28 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>900</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>8</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I7" s="13" t="n">
         <f aca="false">SUM(D5:D7)</f>
@@ -2310,25 +3012,25 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>80</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>8</v>
@@ -2340,25 +3042,25 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>150</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>140</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>16</v>
@@ -2370,25 +3072,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D10" s="11" t="n">
         <v>1400</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>240</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>30</v>
@@ -2400,25 +3102,25 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H11" s="8" t="n">
         <v>1</v>
@@ -2430,25 +3132,25 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D12" s="11" t="n">
         <v>90</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>5.5</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H12" s="8" t="n">
         <v>0.8</v>
@@ -2460,25 +3162,25 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>1200</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>7</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H13" s="8" t="n">
         <v>0.55</v>
@@ -2490,7 +3192,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C15" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D15" s="14" t="n">
         <f aca="false">SUM(D2:D13)</f>
@@ -2525,27 +3227,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>1</v>
@@ -2568,7 +3270,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>2</v>
@@ -2591,7 +3293,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>2</v>
@@ -2614,7 +3316,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>3</v>
@@ -2637,7 +3339,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>4</v>
@@ -2660,7 +3362,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>6</v>
@@ -2683,7 +3385,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>2</v>
@@ -2706,7 +3408,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>1</v>
@@ -2729,29 +3431,29 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B13" s="5" t="n">
         <f aca="false">C2</f>
@@ -2772,7 +3474,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B14" s="5" t="n">
         <f aca="false">D4</f>
@@ -2793,7 +3495,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B15" s="5" t="n">
         <f aca="false">E5</f>
@@ -2814,7 +3516,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -2846,15 +3548,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>9</v>
@@ -2862,7 +3564,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>24</v>
@@ -2870,7 +3572,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>68</v>
@@ -2878,7 +3580,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>165</v>
@@ -2886,36 +3588,36 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="C7" s="7" t="s">
+      <c r="E7" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>154</v>
-      </c>
       <c r="H7" s="7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>2</v>
@@ -2946,7 +3648,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>1</v>
@@ -2977,7 +3679,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>0</v>
@@ -3008,7 +3710,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>0</v>
@@ -3039,7 +3741,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -3076,60 +3778,60 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="G1" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>166</v>
-      </c>
       <c r="H1" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>1</v>
@@ -3175,15 +3877,15 @@
         <v>0.2</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>181</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>1</v>
@@ -3229,15 +3931,15 @@
         <v>0.3</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>1</v>
@@ -3283,15 +3985,15 @@
         <v>0.3</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>1</v>
@@ -3337,15 +4039,15 @@
         <v>2</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>2</v>
@@ -3391,15 +4093,15 @@
         <v>0.6</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>187</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>2</v>
@@ -3445,15 +4147,15 @@
         <v>0.3</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>2</v>
@@ -3499,15 +4201,15 @@
         <v>0.4</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>3</v>
@@ -3553,15 +4255,15 @@
         <v>5</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>4</v>
@@ -3607,17 +4309,17 @@
         <v>0.45</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -3648,27 +4350,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>2</v>
@@ -3691,7 +4393,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>4</v>
@@ -3714,7 +4416,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>5</v>
@@ -3737,7 +4439,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>9</v>
@@ -3760,7 +4462,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>3</v>
@@ -3783,7 +4485,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>1</v>
@@ -3806,7 +4508,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>3</v>
@@ -3829,7 +4531,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>5</v>
@@ -3852,7 +4554,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>8</v>
@@ -3875,7 +4577,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>11</v>
@@ -3898,7 +4600,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>4</v>
@@ -3921,7 +4623,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>10</v>
@@ -3944,7 +4646,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>16</v>
@@ -3967,7 +4669,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>40</v>
@@ -3990,7 +4692,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -4023,37 +4725,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B2" s="5" t="n">
         <f aca="false">Parts!$F$8</f>
         <v>80</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D2" s="19" t="n">
         <f aca="false">Parts!$H$11</f>
@@ -4074,14 +4776,14 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B3" s="5" t="n">
         <f aca="false">Parts!$F$8</f>
         <v>80</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D3" s="19" t="n">
         <f aca="false">Parts!$H$12</f>
@@ -4102,14 +4804,14 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B4" s="5" t="n">
         <f aca="false">Parts!$F$8</f>
         <v>80</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D4" s="19" t="n">
         <f aca="false">Parts!$H$13</f>
@@ -4130,14 +4832,14 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">Parts!$F$9</f>
         <v>140</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D5" s="19" t="n">
         <f aca="false">Parts!$H$11</f>
@@ -4158,14 +4860,14 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">Parts!$F$9</f>
         <v>140</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D6" s="19" t="n">
         <f aca="false">Parts!$H$12</f>
@@ -4186,14 +4888,14 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">Parts!$F$9</f>
         <v>140</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D7" s="19" t="n">
         <f aca="false">Parts!$H$13</f>
@@ -4214,14 +4916,14 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">Parts!$F$10</f>
         <v>240</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">Parts!$H$11</f>
@@ -4242,14 +4944,14 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">Parts!$F$10</f>
         <v>240</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">Parts!$H$12</f>
@@ -4270,14 +4972,14 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Parts!$F$10</f>
         <v>240</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D10" s="19" t="n">
         <f aca="false">Parts!$H$13</f>
@@ -4298,7 +5000,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v0.14 Nano-Bots / Mobile outposts
Nano-bot system has been reworked t add more traits and usage.

job board system added.

outposts are now mobile platforms and are the new entry point to caves.
</commit_message>
<xml_diff>
--- a/docs/balancing.xlsx
+++ b/docs/balancing.xlsx
@@ -24,6 +24,7 @@
     <sheet name="Enemies" sheetId="14" state="visible" r:id="rId16"/>
     <sheet name="Flux upgrades" sheetId="15" state="visible" r:id="rId17"/>
     <sheet name="Contracts" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="Nano-bot crew" sheetId="17" state="visible" r:id="rId19"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -35,9 +36,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="406">
-  <si>
-    <t xml:space="preserve">Bolt &amp; Burrow — balancing sheet (v0.11)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="460">
+  <si>
+    <t xml:space="preserve">Bolt &amp; Burrow — balancing sheet (v0.14)</t>
   </si>
   <si>
     <t xml:space="preserve">A planning copy of the numbers in js/config.js. Changing this sheet does NOT change the game:</t>
@@ -91,6 +92,9 @@
     <t xml:space="preserve">Enemies – enemy and boss stats, and how many seconds each weapon takes to beat them</t>
   </si>
   <si>
+    <t xml:space="preserve">Nano-bot crew – loop times and Flux per minute by path length and chips, other jobs per loop, and the daily bot-cache odds</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dig times – seconds to break each block with each arm tier ("—" = too hard for that tier)</t>
   </si>
   <si>
@@ -1253,6 +1257,165 @@
   </si>
   <si>
     <t xml:space="preserve">Three contracts are picked at random each day (same three all day, new ones at midnight). Tier: 0 = start, 1 = Ember Idol home, 2 = Storm Lens home, 3 = Core Heart home (Rustvale).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loop base (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seconds every loop takes (CREW.loopBase)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per socket (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extra seconds for each socket on the path (CREW.loopPerSocket)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shortest path loop (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A path never loops faster than this before Bus chips: up to 4 sockets loop in 12 s (CREW.pathFloor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No-path loop (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A bot with no path bounces around and works this often, with no chip bonuses (CREW.idleLoop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flux per loop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flux job: Flux each loop (CREW.fluxPerLoop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chip bonus Mk I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Job work added by a matching chip on the path (CREW.chipBonus[0])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chip bonus Mk II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CREW.chipBonus[1] (3 Mk I fuse into 1 Mk II)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chip bonus Overcharged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CREW.chipBonus[2], with a drawback (CHIPS.*.over)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bus speed Mk I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bot speed added by a Bus chip (CREW.busBonus[0])</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Old rate (Flux/min per bot)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What one nano-bot made in v0.13 (the old NANOBOT.fluxPerMin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sockets on path</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loop (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flux/min, no chips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One Flux Amp Mk I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Flux Amps Mk I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bus Mk I + rest Flux Amps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vs old rate (no chips)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 (no path)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With no chips a Flux bot makes 10 Flux a minute (the old rate) on any path of up to 4 sockets, or with no path. Sockets past 4 slow the loop, so a long path only pays off with good chips (Mk II, or a Bus).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other jobs (per loop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With one Mk I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With one Mk II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refine (batches)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best recipe the storage can afford; a bonus is a chance of one more batch. Smelt: 35% double output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repair (hull)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only when damaged. Patch: ×1.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scout (radius, blocks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bonus adds 1.5 blocks per +100%. Scout: +2 and marks gas, vents, unstable rock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Haul (radius, blocks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bonus adds 1.5 blocks per +100%. Magpie grabs in range all the time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guard (damage, Cave 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Damage ×(1 + 0.35 × cave number − 1). Sparky chains 60% to a second enemy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daily bot-cache</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unique chance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CREW.daily.uniqueChance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pity (guaranteed on cache #)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CREW.daily.pity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cache #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chance the first unique comes here</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average caches per unique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days to meet all 8 uniques (no repeats)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A lower bound: a unique you already own becomes an Overcharged chip instead</t>
   </si>
 </sst>
 </file>
@@ -1394,7 +1557,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1488,6 +1651,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1743,7 +1914,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1861,8 +2032,13 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="2" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1892,24 +2068,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B2" s="12" t="n">
         <f aca="false">Parts!D6</f>
@@ -1920,12 +2096,12 @@
         <v>-60</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B3" s="12" t="n">
         <f aca="false">Caves!O2</f>
@@ -1936,12 +2112,12 @@
         <v>-140</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C4" s="12" t="n">
         <f aca="false">Caves!N2</f>
@@ -1952,12 +2128,12 @@
         <v>160</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B5" s="12" t="n">
         <f aca="false">Parts!D3</f>
@@ -1968,12 +2144,12 @@
         <v>40</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B6" s="12" t="n">
         <f aca="false">Parts!D9</f>
@@ -1984,12 +2160,12 @@
         <v>-110</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">Caves!O3</f>
@@ -2003,7 +2179,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C8" s="12" t="n">
         <f aca="false">Caves!N3</f>
@@ -2014,12 +2190,12 @@
         <v>490</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">Parts!D7</f>
@@ -2030,12 +2206,12 @@
         <v>-410</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">Caves!O4</f>
@@ -2049,7 +2225,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">Caves!N4</f>
@@ -2060,12 +2236,12 @@
         <v>1090</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -2101,27 +2277,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>1</v>
@@ -2137,12 +2313,12 @@
         <v>120</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>2</v>
@@ -2158,12 +2334,12 @@
         <v>75</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>3</v>
@@ -2179,12 +2355,12 @@
         <v>50</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>4</v>
@@ -2200,20 +2376,20 @@
         <v>120</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B8" s="2" t="n">
         <f aca="false">$B$12+0</f>
@@ -2222,7 +2398,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B9" s="2" t="n">
         <f aca="false">$B$12+1</f>
@@ -2231,7 +2407,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B10" s="2" t="n">
         <f aca="false">$B$12+2</f>
@@ -2240,7 +2416,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>3</v>
@@ -2248,50 +2424,50 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>1</v>
@@ -2330,7 +2506,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>1</v>
@@ -2369,7 +2545,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>1</v>
@@ -2408,7 +2584,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>2</v>
@@ -2447,7 +2623,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -2479,27 +2655,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>3</v>
@@ -2511,15 +2687,15 @@
         <v>0.3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>1</v>
@@ -2531,15 +2707,15 @@
         <v>0</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2</v>
@@ -2551,15 +2727,15 @@
         <v>0.1</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>3</v>
@@ -2571,35 +2747,35 @@
         <v>0.3</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>
@@ -2635,48 +2811,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C2" s="11" t="n">
         <v>0</v>
@@ -2707,18 +2883,18 @@
         <v>3.33333333333333</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C3" s="11" t="n">
         <v>180</v>
@@ -2749,18 +2925,18 @@
         <v>10.2857142857143</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C4" s="11" t="n">
         <v>220</v>
@@ -2791,18 +2967,18 @@
         <v>2.5</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C5" s="11" t="n">
         <v>260</v>
@@ -2833,18 +3009,18 @@
         <v>0.25</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C6" s="11" t="n">
         <v>300</v>
@@ -2875,18 +3051,18 @@
         <v>0</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>1</v>
@@ -2900,7 +3076,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>1</v>
@@ -2914,7 +3090,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -2949,42 +3125,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>10</v>
@@ -3016,10 +3192,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>338</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>337</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>5</v>
@@ -3051,10 +3227,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>14</v>
@@ -3086,10 +3262,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>22</v>
@@ -3121,10 +3297,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>3</v>
@@ -3156,10 +3332,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>70</v>
@@ -3191,10 +3367,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>160</v>
@@ -3226,10 +3402,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>450</v>
@@ -3261,10 +3437,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>220</v>
@@ -3296,10 +3472,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>300</v>
@@ -3331,10 +3507,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>800</v>
@@ -3366,7 +3542,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -3398,30 +3574,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>0.7</v>
@@ -3441,12 +3617,12 @@
         <v>5</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>15</v>
@@ -3466,12 +3642,12 @@
         <v>135</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>0.06</v>
@@ -3491,12 +3667,12 @@
         <v>0.3</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>0.5</v>
@@ -3516,12 +3692,12 @@
         <v>2.5</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>0.1</v>
@@ -3541,12 +3717,12 @@
         <v>0.5</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>0.08</v>
@@ -3566,12 +3742,12 @@
         <v>0.4</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>1</v>
@@ -3591,21 +3767,21 @@
         <v>5</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3690,7 +3866,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C16" s="13" t="n">
         <f aca="false">C14*7</f>
@@ -3703,7 +3879,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
   </sheetData>
@@ -3735,39 +3911,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>40</v>
@@ -3802,7 +3978,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>8</v>
@@ -3837,7 +4013,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>6</v>
@@ -3872,7 +4048,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
@@ -3907,7 +4083,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>15</v>
@@ -3942,7 +4118,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>2</v>
@@ -3977,7 +4153,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>150</v>
@@ -4012,7 +4188,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>1</v>
@@ -4047,7 +4223,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>20</v>
@@ -4082,7 +4258,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>2</v>
@@ -4117,7 +4293,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -4144,7 +4320,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B15" s="23" t="n">
         <v>2.2</v>
@@ -4152,7 +4328,711 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>405</v>
+        <v>406</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="B15" s="15" t="n">
+        <f aca="false">IF(0=0,$B$5,MAX($B$4,$B$2+$B$3*0))</f>
+        <v>12</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <f aca="false">$B$6*60/B15</f>
+        <v>10</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <f aca="false">IF(0=0,C15,$B$6*(1+$B$7)*60/B15)</f>
+        <v>10</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <f aca="false">IF(0=0,C15,$B$6*(1+0*$B$7)*60/B15)</f>
+        <v>10</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <f aca="false">IF(0&lt;2,E15,$B$6*(1+-1*$B$7)*60/(B15/(1+$B$10)))</f>
+        <v>10</v>
+      </c>
+      <c r="G15" s="22" t="n">
+        <f aca="false">C15/$B$11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <f aca="false">IF(1=0,$B$5,MAX($B$4,$B$2+$B$3*1))</f>
+        <v>12</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <f aca="false">$B$6*60/B16</f>
+        <v>10</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <f aca="false">IF(1=0,C16,$B$6*(1+$B$7)*60/B16)</f>
+        <v>12.5</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <f aca="false">IF(1=0,C16,$B$6*(1+1*$B$7)*60/B16)</f>
+        <v>12.5</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <f aca="false">IF(1&lt;2,E16,$B$6*(1+0*$B$7)*60/(B16/(1+$B$10)))</f>
+        <v>12.5</v>
+      </c>
+      <c r="G16" s="22" t="n">
+        <f aca="false">C16/$B$11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="15" t="n">
+        <f aca="false">IF(2=0,$B$5,MAX($B$4,$B$2+$B$3*2))</f>
+        <v>12</v>
+      </c>
+      <c r="C17" s="15" t="n">
+        <f aca="false">$B$6*60/B17</f>
+        <v>10</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <f aca="false">IF(2=0,C17,$B$6*(1+$B$7)*60/B17)</f>
+        <v>12.5</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <f aca="false">IF(2=0,C17,$B$6*(1+2*$B$7)*60/B17)</f>
+        <v>15</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <f aca="false">IF(2&lt;2,E17,$B$6*(1+1*$B$7)*60/(B17/(1+$B$10)))</f>
+        <v>14.375</v>
+      </c>
+      <c r="G17" s="22" t="n">
+        <f aca="false">C17/$B$11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="15" t="n">
+        <f aca="false">IF(3=0,$B$5,MAX($B$4,$B$2+$B$3*3))</f>
+        <v>12</v>
+      </c>
+      <c r="C18" s="15" t="n">
+        <f aca="false">$B$6*60/B18</f>
+        <v>10</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <f aca="false">IF(3=0,C18,$B$6*(1+$B$7)*60/B18)</f>
+        <v>12.5</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <f aca="false">IF(3=0,C18,$B$6*(1+3*$B$7)*60/B18)</f>
+        <v>17.5</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <f aca="false">IF(3&lt;2,E18,$B$6*(1+2*$B$7)*60/(B18/(1+$B$10)))</f>
+        <v>17.25</v>
+      </c>
+      <c r="G18" s="22" t="n">
+        <f aca="false">C18/$B$11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="15" t="n">
+        <f aca="false">IF(4=0,$B$5,MAX($B$4,$B$2+$B$3*4))</f>
+        <v>12</v>
+      </c>
+      <c r="C19" s="15" t="n">
+        <f aca="false">$B$6*60/B19</f>
+        <v>10</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <f aca="false">IF(4=0,C19,$B$6*(1+$B$7)*60/B19)</f>
+        <v>12.5</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <f aca="false">IF(4=0,C19,$B$6*(1+4*$B$7)*60/B19)</f>
+        <v>20</v>
+      </c>
+      <c r="F19" s="15" t="n">
+        <f aca="false">IF(4&lt;2,E19,$B$6*(1+3*$B$7)*60/(B19/(1+$B$10)))</f>
+        <v>20.125</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <f aca="false">C19/$B$11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" s="15" t="n">
+        <f aca="false">IF(5=0,$B$5,MAX($B$4,$B$2+$B$3*5))</f>
+        <v>13.5</v>
+      </c>
+      <c r="C20" s="15" t="n">
+        <f aca="false">$B$6*60/B20</f>
+        <v>8.88888888888889</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <f aca="false">IF(5=0,C20,$B$6*(1+$B$7)*60/B20)</f>
+        <v>11.1111111111111</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <f aca="false">IF(5=0,C20,$B$6*(1+5*$B$7)*60/B20)</f>
+        <v>20</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <f aca="false">IF(5&lt;2,E20,$B$6*(1+4*$B$7)*60/(B20/(1+$B$10)))</f>
+        <v>20.4444444444444</v>
+      </c>
+      <c r="G20" s="22" t="n">
+        <f aca="false">C20/$B$11</f>
+        <v>0.888888888888889</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" s="15" t="n">
+        <f aca="false">IF(6=0,$B$5,MAX($B$4,$B$2+$B$3*6))</f>
+        <v>15</v>
+      </c>
+      <c r="C21" s="15" t="n">
+        <f aca="false">$B$6*60/B21</f>
+        <v>8</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <f aca="false">IF(6=0,C21,$B$6*(1+$B$7)*60/B21)</f>
+        <v>10</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <f aca="false">IF(6=0,C21,$B$6*(1+6*$B$7)*60/B21)</f>
+        <v>20</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <f aca="false">IF(6&lt;2,E21,$B$6*(1+5*$B$7)*60/(B21/(1+$B$10)))</f>
+        <v>20.7</v>
+      </c>
+      <c r="G21" s="22" t="n">
+        <f aca="false">C21/$B$11</f>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" s="15" t="n">
+        <f aca="false">IF(7=0,$B$5,MAX($B$4,$B$2+$B$3*7))</f>
+        <v>16.5</v>
+      </c>
+      <c r="C22" s="15" t="n">
+        <f aca="false">$B$6*60/B22</f>
+        <v>7.27272727272727</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <f aca="false">IF(7=0,C22,$B$6*(1+$B$7)*60/B22)</f>
+        <v>9.09090909090909</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <f aca="false">IF(7=0,C22,$B$6*(1+7*$B$7)*60/B22)</f>
+        <v>20</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <f aca="false">IF(7&lt;2,E22,$B$6*(1+6*$B$7)*60/(B22/(1+$B$10)))</f>
+        <v>20.9090909090909</v>
+      </c>
+      <c r="G22" s="22" t="n">
+        <f aca="false">C22/$B$11</f>
+        <v>0.727272727272727</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" s="15" t="n">
+        <f aca="false">IF(8=0,$B$5,MAX($B$4,$B$2+$B$3*8))</f>
+        <v>18</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <f aca="false">$B$6*60/B23</f>
+        <v>6.66666666666667</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <f aca="false">IF(8=0,C23,$B$6*(1+$B$7)*60/B23)</f>
+        <v>8.33333333333333</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <f aca="false">IF(8=0,C23,$B$6*(1+8*$B$7)*60/B23)</f>
+        <v>20</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <f aca="false">IF(8&lt;2,E23,$B$6*(1+7*$B$7)*60/(B23/(1+$B$10)))</f>
+        <v>21.0833333333333</v>
+      </c>
+      <c r="G23" s="22" t="n">
+        <f aca="false">C23/$B$11</f>
+        <v>0.666666666666667</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="24" t="n">
+        <f aca="false">B28*(1+$B$7)</f>
+        <v>1.25</v>
+      </c>
+      <c r="D28" s="24" t="n">
+        <f aca="false">B28*(1+$B$8)</f>
+        <v>1.6</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="24" t="n">
+        <f aca="false">B29*(1+$B$7)</f>
+        <v>3.75</v>
+      </c>
+      <c r="D29" s="24" t="n">
+        <f aca="false">B29*(1+$B$8)</f>
+        <v>4.8</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="15" t="n">
+        <f aca="false">B30+1.5*$B$7</f>
+        <v>4.375</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <f aca="false">B30+1.5*$B$8</f>
+        <v>4.9</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="15" t="n">
+        <f aca="false">B31+1.5*$B$7</f>
+        <v>4.375</v>
+      </c>
+      <c r="D31" s="15" t="n">
+        <f aca="false">B31+1.5*$B$8</f>
+        <v>4.9</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C32" s="24" t="n">
+        <f aca="false">B32*(1+$B$7)</f>
+        <v>3.125</v>
+      </c>
+      <c r="D32" s="24" t="n">
+        <f aca="false">B32*(1+$B$8)</f>
+        <v>4</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="B36" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="25" t="n">
+        <f aca="false">IF(A40&lt;$B$37,(1-$B$36)^(A40-1)*$B$36,(1-$B$36)^($B$37-1))</f>
+        <v>0.2</v>
+      </c>
+      <c r="C40" s="25" t="n">
+        <f aca="false">SUM($B$40:B40)</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="25" t="n">
+        <f aca="false">IF(A41&lt;$B$37,(1-$B$36)^(A41-1)*$B$36,(1-$B$36)^($B$37-1))</f>
+        <v>0.16</v>
+      </c>
+      <c r="C41" s="25" t="n">
+        <f aca="false">SUM($B$40:B41)</f>
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" s="25" t="n">
+        <f aca="false">IF(A42&lt;$B$37,(1-$B$36)^(A42-1)*$B$36,(1-$B$36)^($B$37-1))</f>
+        <v>0.128</v>
+      </c>
+      <c r="C42" s="25" t="n">
+        <f aca="false">SUM($B$40:B42)</f>
+        <v>0.488</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="25" t="n">
+        <f aca="false">IF(A43&lt;$B$37,(1-$B$36)^(A43-1)*$B$36,(1-$B$36)^($B$37-1))</f>
+        <v>0.1024</v>
+      </c>
+      <c r="C43" s="25" t="n">
+        <f aca="false">SUM($B$40:B43)</f>
+        <v>0.5904</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B44" s="25" t="n">
+        <f aca="false">IF(A44&lt;$B$37,(1-$B$36)^(A44-1)*$B$36,(1-$B$36)^($B$37-1))</f>
+        <v>0.08192</v>
+      </c>
+      <c r="C44" s="25" t="n">
+        <f aca="false">SUM($B$40:B44)</f>
+        <v>0.67232</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B45" s="25" t="n">
+        <f aca="false">IF(A45&lt;$B$37,(1-$B$36)^(A45-1)*$B$36,(1-$B$36)^($B$37-1))</f>
+        <v>0.065536</v>
+      </c>
+      <c r="C45" s="25" t="n">
+        <f aca="false">SUM($B$40:B45)</f>
+        <v>0.737856</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B46" s="25" t="n">
+        <f aca="false">IF(A46&lt;$B$37,(1-$B$36)^(A46-1)*$B$36,(1-$B$36)^($B$37-1))</f>
+        <v>0.262144</v>
+      </c>
+      <c r="C46" s="25" t="n">
+        <f aca="false">SUM($B$40:B46)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="B48" s="24" t="n">
+        <f aca="false">SUMPRODUCT(A40:A46,B40:B46)</f>
+        <v>3.951424</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="B49" s="17" t="n">
+        <f aca="false">B48*8</f>
+        <v>31.611392</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>459</v>
       </c>
     </row>
   </sheetData>
@@ -4181,244 +5061,244 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>1.2</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>45</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>80</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>60</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>160</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>54</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>0.5</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>0.4</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>1.8</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>0.25</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>0.3</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B22" s="4" t="n">
         <v>75</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -4457,61 +5337,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="S1" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4519,19 +5399,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E2" s="10" t="n">
         <v>0.06</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G2" s="10" t="n">
         <v>0.025</v>
@@ -4552,7 +5432,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="N2" s="11" t="n">
         <v>300</v>
@@ -4573,7 +5453,7 @@
         <v>160</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4581,19 +5461,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C3" s="9" t="n">
         <v>1.5</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E3" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G3" s="10" t="n">
         <v>0.03</v>
@@ -4614,7 +5494,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="N3" s="11" t="n">
         <v>800</v>
@@ -4635,7 +5515,7 @@
         <v>240</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4643,19 +5523,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C4" s="9" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G4" s="10" t="n">
         <v>0.025</v>
@@ -4676,7 +5556,7 @@
         <v>3</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="N4" s="11" t="n">
         <v>2000</v>
@@ -4697,7 +5577,7 @@
         <v>320</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4705,19 +5585,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>2.2</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>0.045</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G5" s="10" t="n">
         <v>0.02</v>
@@ -4738,7 +5618,7 @@
         <v>1</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N5" s="11" t="n">
         <v>2500</v>
@@ -4759,7 +5639,7 @@
         <v>352</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4767,19 +5647,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C6" s="9" t="n">
         <v>2.6</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>0.045</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G6" s="10" t="n">
         <v>0.015</v>
@@ -4800,7 +5680,7 @@
         <v>2</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="N6" s="11" t="n">
         <v>4000</v>
@@ -4821,7 +5701,7 @@
         <v>416</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4829,19 +5709,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>3</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G7" s="10" t="n">
         <v>0.035</v>
@@ -4862,7 +5742,7 @@
         <v>2</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="N7" s="11" t="n">
         <v>6000</v>
@@ -4883,22 +5763,22 @@
         <v>480</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -4933,54 +5813,54 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D2" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>2.5</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>0</v>
@@ -4992,25 +5872,25 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D3" s="11" t="n">
         <v>120</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>3</v>
@@ -5022,25 +5902,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>1000</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>6</v>
@@ -5052,28 +5932,28 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I5" s="13" t="n">
         <f aca="false">SUM(D5:D5)</f>
@@ -5082,28 +5962,28 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>60</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I6" s="13" t="n">
         <f aca="false">SUM(D5:D6)</f>
@@ -5112,28 +5992,28 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>900</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>8</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I7" s="13" t="n">
         <f aca="false">SUM(D5:D7)</f>
@@ -5142,25 +6022,25 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>80</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>8</v>
@@ -5172,25 +6052,25 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>150</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>140</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>16</v>
@@ -5202,25 +6082,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D10" s="11" t="n">
         <v>1400</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>240</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>30</v>
@@ -5232,25 +6112,25 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H11" s="8" t="n">
         <v>1</v>
@@ -5262,25 +6142,25 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D12" s="11" t="n">
         <v>90</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>5.5</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H12" s="8" t="n">
         <v>0.8</v>
@@ -5292,25 +6172,25 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>1200</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>7</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H13" s="8" t="n">
         <v>0.55</v>
@@ -5322,7 +6202,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C15" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D15" s="14" t="n">
         <f aca="false">SUM(D2:D13)</f>
@@ -5357,27 +6237,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>1</v>
@@ -5400,7 +6280,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>2</v>
@@ -5423,7 +6303,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>2</v>
@@ -5446,7 +6326,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>3</v>
@@ -5469,7 +6349,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>4</v>
@@ -5492,7 +6372,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>6</v>
@@ -5515,7 +6395,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>2</v>
@@ -5538,7 +6418,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>1</v>
@@ -5561,29 +6441,29 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B13" s="5" t="n">
         <f aca="false">C2</f>
@@ -5604,7 +6484,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B14" s="5" t="n">
         <f aca="false">D4</f>
@@ -5625,7 +6505,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B15" s="5" t="n">
         <f aca="false">E5</f>
@@ -5646,7 +6526,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -5678,15 +6558,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>9</v>
@@ -5694,7 +6574,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>24</v>
@@ -5702,7 +6582,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>68</v>
@@ -5710,7 +6590,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>165</v>
@@ -5718,36 +6598,36 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="F7" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>166</v>
-      </c>
       <c r="H7" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>2</v>
@@ -5778,7 +6658,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>1</v>
@@ -5809,7 +6689,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>0</v>
@@ -5840,7 +6720,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>0</v>
@@ -5871,7 +6751,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -5908,60 +6788,60 @@
   <sheetData>
     <row r="1" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>1</v>
@@ -6007,15 +6887,15 @@
         <v>0.2</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>1</v>
@@ -6061,15 +6941,15 @@
         <v>0.3</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>1</v>
@@ -6115,15 +6995,15 @@
         <v>0.3</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>1</v>
@@ -6169,15 +7049,15 @@
         <v>2</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>2</v>
@@ -6223,15 +7103,15 @@
         <v>0.6</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>2</v>
@@ -6277,15 +7157,15 @@
         <v>0.3</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>2</v>
@@ -6331,15 +7211,15 @@
         <v>0.4</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>3</v>
@@ -6385,15 +7265,15 @@
         <v>5</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>4</v>
@@ -6439,17 +7319,17 @@
         <v>0.45</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -6480,27 +7360,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>2</v>
@@ -6523,7 +7403,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>4</v>
@@ -6546,7 +7426,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>5</v>
@@ -6569,7 +7449,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>9</v>
@@ -6592,7 +7472,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>3</v>
@@ -6615,7 +7495,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>1</v>
@@ -6638,7 +7518,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>3</v>
@@ -6661,7 +7541,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>5</v>
@@ -6684,7 +7564,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>8</v>
@@ -6707,7 +7587,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>11</v>
@@ -6730,7 +7610,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>4</v>
@@ -6753,7 +7633,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>10</v>
@@ -6776,7 +7656,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>16</v>
@@ -6799,7 +7679,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>40</v>
@@ -6822,7 +7702,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -6855,37 +7735,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B2" s="5" t="n">
         <f aca="false">Parts!$F$8</f>
         <v>80</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D2" s="19" t="n">
         <f aca="false">Parts!$H$11</f>
@@ -6906,14 +7786,14 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B3" s="5" t="n">
         <f aca="false">Parts!$F$8</f>
         <v>80</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D3" s="19" t="n">
         <f aca="false">Parts!$H$12</f>
@@ -6934,14 +7814,14 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B4" s="5" t="n">
         <f aca="false">Parts!$F$8</f>
         <v>80</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D4" s="19" t="n">
         <f aca="false">Parts!$H$13</f>
@@ -6962,14 +7842,14 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">Parts!$F$9</f>
         <v>140</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D5" s="19" t="n">
         <f aca="false">Parts!$H$11</f>
@@ -6990,14 +7870,14 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">Parts!$F$9</f>
         <v>140</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D6" s="19" t="n">
         <f aca="false">Parts!$H$12</f>
@@ -7018,14 +7898,14 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">Parts!$F$9</f>
         <v>140</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D7" s="19" t="n">
         <f aca="false">Parts!$H$13</f>
@@ -7046,14 +7926,14 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">Parts!$F$10</f>
         <v>240</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D8" s="19" t="n">
         <f aca="false">Parts!$H$11</f>
@@ -7074,14 +7954,14 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">Parts!$F$10</f>
         <v>240</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">Parts!$H$12</f>
@@ -7102,14 +7982,14 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Parts!$F$10</f>
         <v>240</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D10" s="19" t="n">
         <f aca="false">Parts!$H$13</f>
@@ -7130,7 +8010,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>